<commit_message>
adjusted positive test case to include a 'has_no_data' test
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/positive/01/data/new-rule-positive-01.xlsx
+++ b/rules/NEW-RULE/positive/01/data/new-rule-positive-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/positive/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F10155EE-D659-1A4A-BF74-1D0D9BFE67ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{618545CC-A684-D04C-AD3A-5458C4E3C3B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="71">
   <si>
     <t>Product</t>
   </si>
@@ -157,6 +157,9 @@
     <t>CDISC001</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
@@ -169,9 +172,6 @@
     <t>-28</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>2</t>
   </si>
   <si>
@@ -185,9 +185,6 @@
   </si>
   <si>
     <t>DAY 2</t>
-  </si>
-  <si>
-    <t>YES</t>
   </si>
   <si>
     <t>4</t>
@@ -278,7 +275,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
-        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -298,9 +294,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -747,7 +741,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="64" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>22</v>
       </c>
@@ -785,7 +779,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>34</v>
       </c>
@@ -823,7 +817,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>12</v>
       </c>
@@ -871,31 +865,31 @@
       <c r="C5" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D5" s="1"/>
+      <c r="D5" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="E5" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="K5" s="1">
         <v>1</v>
       </c>
-      <c r="L5" s="1" t="s">
-        <v>48</v>
-      </c>
+      <c r="L5" s="1"/>
     </row>
     <row r="6" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
@@ -907,7 +901,9 @@
       <c r="C6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="1"/>
+      <c r="D6" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="E6" s="1" t="s">
         <v>49</v>
       </c>
@@ -915,7 +911,7 @@
         <v>50</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>51</v>
@@ -924,14 +920,12 @@
         <v>51</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>48</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="L6" s="1"/>
     </row>
     <row r="7" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
@@ -943,7 +937,9 @@
       <c r="C7" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="1"/>
+      <c r="D7" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="E7" s="1" t="s">
         <v>52</v>
       </c>
@@ -951,23 +947,21 @@
         <v>53</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>54</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="L7" s="1"/>
     </row>
     <row r="8" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
@@ -979,12 +973,14 @@
       <c r="C8" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="1"/>
+      <c r="D8" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="E8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>56</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>37</v>
@@ -993,23 +989,20 @@
         <v>38</v>
       </c>
       <c r="I8" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="K8" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>48</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="L8" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L4 A5:C8 E5:L8" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L4 A8:K8 A7:K7 A6:K6 A5:K5" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1033,16 +1026,16 @@
         <v>15</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="48" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>22</v>
       </c>
@@ -1056,16 +1049,16 @@
         <v>27</v>
       </c>
       <c r="E2" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>34</v>
       </c>
@@ -1088,7 +1081,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>12</v>
       </c>
@@ -1099,16 +1092,16 @@
         <v>38</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -1116,22 +1109,22 @@
         <v>41</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>68</v>
-      </c>
       <c r="G5" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -1139,20 +1132,22 @@
         <v>41</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D6" s="1"/>
+      <c r="D6" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="E6" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -1160,22 +1155,22 @@
         <v>41</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>52</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.2">
@@ -1183,28 +1178,28 @@
         <v>41</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>67</v>
-      </c>
       <c r="F8" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:G5 A7:G8 A6:C6 E6:G6" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:G8" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Bugfix - included match datasets info in the YAML file and corrected one value in one Excel file
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/positive/01/data/new-rule-positive-01.xlsx
+++ b/rules/NEW-RULE/positive/01/data/new-rule-positive-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/positive/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241BD48C-2FAC-ED46-AD83-5B3DD0C3686D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C0E1BDC-70E9-4E48-BED1-0CF59552A6CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -711,7 +711,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -720,8 +720,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1428,10 +1427,10 @@
       <c r="F5" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="8" t="s">
         <v>159</v>
       </c>
       <c r="I5" s="3" t="s">
@@ -1502,10 +1501,10 @@
       <c r="F6" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="8" t="s">
         <v>164</v>
       </c>
       <c r="I6" s="3" t="s">
@@ -1578,10 +1577,10 @@
       <c r="F7" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="8" t="s">
         <v>166</v>
       </c>
       <c r="I7" s="3" t="s">
@@ -1652,10 +1651,10 @@
       <c r="F8" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="8" t="s">
         <v>171</v>
       </c>
       <c r="I8" s="3" t="s">
@@ -1720,10 +1719,10 @@
       <c r="F9" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="8" t="s">
         <v>173</v>
       </c>
       <c r="I9" s="3" t="s">
@@ -1792,10 +1791,10 @@
       <c r="F10" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="8" t="s">
         <v>157</v>
       </c>
       <c r="I10" s="3" t="s">
@@ -1860,10 +1859,10 @@
       <c r="F11" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="8" t="s">
         <v>179</v>
       </c>
       <c r="I11" s="3" t="s">
@@ -1934,10 +1933,10 @@
       <c r="F12" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="H12" s="8" t="s">
         <v>183</v>
       </c>
       <c r="I12" s="3" t="s">
@@ -2010,10 +2009,10 @@
       <c r="F13" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="H13" s="8" t="s">
         <v>153</v>
       </c>
       <c r="I13" s="3" t="s">
@@ -2084,10 +2083,10 @@
       <c r="F14" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="H14" s="8" t="s">
         <v>187</v>
       </c>
       <c r="I14" s="3" t="s">
@@ -2449,7 +2448,7 @@
       <c r="Q5" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="R5" s="3" t="s">
+      <c r="R5" s="8" t="s">
         <v>138</v>
       </c>
       <c r="S5" s="3">
@@ -2511,7 +2510,7 @@
       <c r="Q6" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="R6" s="3" t="s">
+      <c r="R6" s="8" t="s">
         <v>139</v>
       </c>
       <c r="S6" s="3">
@@ -2573,7 +2572,7 @@
       <c r="Q7" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="R7" s="3" t="s">
+      <c r="R7" s="8" t="s">
         <v>140</v>
       </c>
       <c r="S7" s="3">
@@ -2635,7 +2634,7 @@
       <c r="Q8" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="R8" s="3" t="s">
+      <c r="R8" s="8" t="s">
         <v>141</v>
       </c>
       <c r="S8" s="3">
@@ -2697,7 +2696,7 @@
       <c r="Q9" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="R9" s="3" t="s">
+      <c r="R9" s="8" t="s">
         <v>142</v>
       </c>
       <c r="S9" s="3">
@@ -2759,7 +2758,7 @@
       <c r="Q10" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="R10" s="3" t="s">
+      <c r="R10" s="8" t="s">
         <v>143</v>
       </c>
       <c r="S10" s="3">
@@ -2821,7 +2820,7 @@
       <c r="Q11" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="R11" s="3" t="s">
+      <c r="R11" s="8" t="s">
         <v>144</v>
       </c>
       <c r="S11" s="3">
@@ -2883,7 +2882,7 @@
       <c r="Q12" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="R12" s="3" t="s">
+      <c r="R12" s="8" t="s">
         <v>145</v>
       </c>
       <c r="S12" s="3">
@@ -2945,7 +2944,7 @@
       <c r="Q13" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="R13" s="3" t="s">
+      <c r="R13" s="8" t="s">
         <v>146</v>
       </c>
       <c r="S13" s="3">
@@ -3007,7 +3006,7 @@
       <c r="Q14" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="R14" s="3" t="s">
+      <c r="R14" s="8" t="s">
         <v>147</v>
       </c>
       <c r="S14" s="3">
@@ -3069,7 +3068,7 @@
       <c r="Q15" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="R15" s="3" t="s">
+      <c r="R15" s="8" t="s">
         <v>150</v>
       </c>
       <c r="S15" s="3">
@@ -3131,7 +3130,7 @@
       <c r="Q16" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="R16" s="3" t="s">
+      <c r="R16" s="8" t="s">
         <v>151</v>
       </c>
       <c r="S16" s="3">
@@ -3193,7 +3192,7 @@
       <c r="Q17" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="R17" s="3" t="s">
+      <c r="R17" s="8" t="s">
         <v>152</v>
       </c>
       <c r="S17" s="3">
@@ -3255,7 +3254,7 @@
       <c r="Q18" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="R18" s="3" t="s">
+      <c r="R18" s="8" t="s">
         <v>154</v>
       </c>
       <c r="S18" s="3">
@@ -3317,7 +3316,7 @@
       <c r="Q19" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="R19" s="3" t="s">
+      <c r="R19" s="8" t="s">
         <v>155</v>
       </c>
       <c r="S19" s="3">
@@ -3379,7 +3378,7 @@
       <c r="Q20" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="R20" s="3" t="s">
+      <c r="R20" s="8" t="s">
         <v>158</v>
       </c>
       <c r="S20" s="3">

</xml_diff>

<commit_message>
expanded and improved test cases
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/positive/01/data/new-rule-positive-01.xlsx
+++ b/rules/NEW-RULE/positive/01/data/new-rule-positive-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/positive/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{380B7BE0-9E34-904A-9921-03F3B6D9DF60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF2B8CE6-9B8F-2548-A45B-F38E74D80E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-4560" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="204">
   <si>
     <t>Product</t>
   </si>
@@ -631,6 +631,9 @@
   </si>
   <si>
     <t>NA</t>
+  </si>
+  <si>
+    <t>AD</t>
   </si>
 </sst>
 </file>
@@ -722,7 +725,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1079,7 +1082,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:11" ht="32" x14ac:dyDescent="0.2">
@@ -1618,7 +1621,9 @@
       <c r="C21" s="4">
         <v>1</v>
       </c>
-      <c r="D21" s="4"/>
+      <c r="D21" s="4" t="s">
+        <v>120</v>
+      </c>
       <c r="E21" s="4" t="s">
         <v>88</v>
       </c>
@@ -1639,94 +1644,107 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="80" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="4">
-        <v>1</v>
+      <c r="C22" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>122</v>
       </c>
       <c r="E22" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="80" x14ac:dyDescent="0.2">
+      <c r="A23" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" s="4">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F23" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G23" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="80" x14ac:dyDescent="0.2">
+      <c r="A24" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="G24" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="H22" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="I22" s="4" t="s">
+      <c r="H24" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="I24" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="J22" s="4" t="s">
+      <c r="J24" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="K22" s="4" t="s">
+      <c r="K24" s="4" t="s">
         <v>95</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A23" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C23" s="4">
-        <v>1</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="I23" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="J23" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K23" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A24" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="4">
-        <v>1</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="J24" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K24" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="32" x14ac:dyDescent="0.2">
@@ -1740,85 +1758,97 @@
         <v>1</v>
       </c>
       <c r="E25" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A26" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" s="4">
+        <v>1</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C27" s="4">
+        <v>1</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F27" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G27" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="J25" s="4" t="s">
+      <c r="J27" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C26" s="4">
-        <v>1</v>
-      </c>
-      <c r="E26" s="4" t="s">
+    <row r="28" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A28" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" s="4">
+        <v>1</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F28" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G28" s="4" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="112" x14ac:dyDescent="0.2">
-      <c r="A27" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C27" s="4">
-        <v>1</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="112" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C28" s="4">
-        <v>2</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>31</v>
       </c>
@@ -1832,16 +1862,16 @@
         <v>109</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="365" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>31</v>
       </c>
@@ -1852,27 +1882,27 @@
         <v>2</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="335" x14ac:dyDescent="0.2">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C31" s="4" t="s">
-        <v>70</v>
+      <c r="C31" s="4">
+        <v>1</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>109</v>
@@ -1884,21 +1914,21 @@
         <v>116</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" ht="128" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="365" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C32" s="4" t="s">
-        <v>120</v>
+      <c r="C32" s="4">
+        <v>2</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>115</v>
@@ -1907,10 +1937,10 @@
         <v>116</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" ht="112" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="335" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>31</v>
       </c>
@@ -1918,10 +1948,10 @@
         <v>32</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>122</v>
+        <v>70</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>115</v>
@@ -1930,128 +1960,128 @@
         <v>116</v>
       </c>
       <c r="G33" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="128" x14ac:dyDescent="0.2">
+      <c r="A34" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="112" x14ac:dyDescent="0.2">
+      <c r="A35" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="G35" s="4" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="64" x14ac:dyDescent="0.2">
-      <c r="A34" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C34" s="4">
-        <v>1</v>
-      </c>
-      <c r="E34" s="4" t="s">
+    <row r="36" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+      <c r="A36" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C36" s="4">
+        <v>1</v>
+      </c>
+      <c r="E36" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="F36" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="G34" s="4" t="s">
+      <c r="G36" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="I34" s="4" t="s">
+      <c r="I36" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="J34" s="4" t="s">
+      <c r="J36" s="4" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="64" x14ac:dyDescent="0.2">
-      <c r="A35" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" s="4">
-        <v>1</v>
-      </c>
-      <c r="E35" s="4" t="s">
+    <row r="37" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37" s="4">
+        <v>1</v>
+      </c>
+      <c r="E37" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="F37" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="G35" s="4" t="s">
+      <c r="G37" s="4" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A36" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C36" s="4">
-        <v>1</v>
-      </c>
-      <c r="E36" s="4" t="s">
+    <row r="38" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A38" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" s="4">
+        <v>1</v>
+      </c>
+      <c r="E38" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="F38" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="G36" s="4" t="s">
+      <c r="G38" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="I36" s="4" t="s">
+      <c r="I38" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="J36" s="4" t="s">
+      <c r="J38" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K36" s="4" t="s">
+      <c r="K38" s="4" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A37" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C37" s="4">
-        <v>1</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="F37" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="G37" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A38" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C38" s="4">
-        <v>1</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="G38" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="I38" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="J38" s="4" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="48" x14ac:dyDescent="0.2">
@@ -2065,22 +2095,13 @@
         <v>1</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="I39" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="J39" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K39" s="4" t="s">
-        <v>41</v>
+        <v>136</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="32" x14ac:dyDescent="0.2">
@@ -2094,16 +2115,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="J40" s="4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>31</v>
       </c>
@@ -2114,13 +2141,22 @@
         <v>1</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>150</v>
+        <v>143</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="J41" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K41" s="4" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="32" x14ac:dyDescent="0.2">
@@ -2134,108 +2170,105 @@
         <v>1</v>
       </c>
       <c r="E42" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A43" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C43" s="4">
+        <v>1</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A44" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C44" s="4">
+        <v>1</v>
+      </c>
+      <c r="E44" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="F42" s="4" t="s">
+      <c r="F44" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="G42" s="4" t="s">
+      <c r="G44" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="J42" s="4" t="s">
+      <c r="J44" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A43" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C43" s="4">
-        <v>1</v>
-      </c>
-      <c r="E43" s="4" t="s">
+    <row r="45" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A45" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C45" s="4">
+        <v>1</v>
+      </c>
+      <c r="E45" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="F43" s="4" t="s">
+      <c r="F45" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="G43" s="4" t="s">
+      <c r="G45" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="I43" s="4" t="s">
+      <c r="I45" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="J43" s="4" t="s">
+      <c r="J45" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K43" s="4" t="s">
+      <c r="K45" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="96" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C44" s="4">
-        <v>1</v>
-      </c>
-      <c r="E44" s="4" t="s">
+    <row r="46" spans="1:11" ht="96" x14ac:dyDescent="0.2">
+      <c r="A46" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C46" s="4">
+        <v>1</v>
+      </c>
+      <c r="E46" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="F44" s="4" t="s">
+      <c r="F46" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="G44" s="4" t="s">
+      <c r="G46" s="4" t="s">
         <v>160</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A45" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C45" s="4">
-        <v>1</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="F45" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="G45" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="J45" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A46" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C46" s="4">
-        <v>1</v>
-      </c>
-      <c r="E46" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="F46" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="G46" s="4" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="32" x14ac:dyDescent="0.2">
@@ -2249,22 +2282,16 @@
         <v>1</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="I47" s="4" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K47" s="4" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="48" x14ac:dyDescent="0.2">
@@ -2278,22 +2305,13 @@
         <v>1</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="I48" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="J48" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K48" s="4" t="s">
-        <v>41</v>
+        <v>166</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="32" x14ac:dyDescent="0.2">
@@ -2307,16 +2325,16 @@
         <v>1</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>63</v>
+        <v>169</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="J49" s="4" t="s">
         <v>40</v>
@@ -2325,7 +2343,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="112" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>31</v>
       </c>
@@ -2336,20 +2354,25 @@
         <v>1</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="H50" s="4"/>
-      <c r="I50" s="4"/>
-      <c r="J50" s="4"/>
-      <c r="K50" s="4"/>
-    </row>
-    <row r="51" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+        <v>173</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="J50" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K50" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>31</v>
       </c>
@@ -2360,16 +2383,16 @@
         <v>1</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>183</v>
+        <v>63</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="J51" s="4" t="s">
         <v>40</v>
@@ -2378,7 +2401,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="160" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>31</v>
       </c>
@@ -2389,16 +2412,20 @@
         <v>1</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+        <v>180</v>
+      </c>
+      <c r="H52" s="4"/>
+      <c r="I52" s="4"/>
+      <c r="J52" s="4"/>
+      <c r="K52" s="4"/>
+    </row>
+    <row r="53" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
         <v>31</v>
       </c>
@@ -2409,16 +2436,16 @@
         <v>1</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="J53" s="4" t="s">
         <v>40</v>
@@ -2427,7 +2454,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="96" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11" ht="160" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>31</v>
       </c>
@@ -2438,22 +2465,16 @@
         <v>1</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="I54" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="J54" s="4" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>31</v>
       </c>
@@ -2464,16 +2485,16 @@
         <v>1</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>113</v>
+        <v>190</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="J55" s="4" t="s">
         <v>40</v>
@@ -2482,32 +2503,87 @@
         <v>41</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C56" s="4" t="s">
+      <c r="C56" s="4">
+        <v>1</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="I56" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="J56" s="4" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A57" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C57" s="4">
+        <v>1</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="I57" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="J57" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K57" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A58" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C58" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="E56" s="4" t="s">
+      <c r="E58" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="F56" s="4" t="s">
+      <c r="F58" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="G56" s="4" t="s">
+      <c r="G58" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="I56" s="4" t="s">
+      <c r="I58" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="J56" s="4" t="s">
+      <c r="J58" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K56" s="4" t="s">
+      <c r="K58" s="4" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>

<commit_message>
matched PC and PP directly and fixed validation output
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/positive/01/data/new-rule-positive-01.xlsx
+++ b/rules/NEW-RULE/positive/01/data/new-rule-positive-01.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enrico/Work/core-contributor/rules/NEW-RULE/positive/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A7537C1-7054-D540-A256-1C65524BF887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E2423F8-D0A2-614F-91EA-C00FF827F37F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30240" yWindow="-7000" windowWidth="51200" windowHeight="28800" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,13 @@
     <sheet name="Datasets" sheetId="2" r:id="rId2"/>
     <sheet name="pc.xpt" sheetId="4" r:id="rId3"/>
     <sheet name="pp.xpt" sheetId="3" r:id="rId4"/>
-    <sheet name="relrec.xpt" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="99">
   <si>
     <t>Product</t>
   </si>
@@ -92,9 +91,6 @@
     <t>PCORRESU</t>
   </si>
   <si>
-    <t>8</t>
-  </si>
-  <si>
     <t>PC</t>
   </si>
   <si>
@@ -315,44 +311,6 @@
   </si>
   <si>
     <t>123-0002-13</t>
-  </si>
-  <si>
-    <t>RDOMAIN</t>
-  </si>
-  <si>
-    <t>IDVAR</t>
-  </si>
-  <si>
-    <t>IDVARVAL</t>
-  </si>
-  <si>
-    <t>RELTYPE</t>
-  </si>
-  <si>
-    <t>RELID</t>
-  </si>
-  <si>
-    <t>Identifying
-Variable</t>
-  </si>
-  <si>
-    <t>Identifying
-VariableValue</t>
-  </si>
-  <si>
-    <t>RelationshipType</t>
-  </si>
-  <si>
-    <t>RelationshipIdentifier</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>ONE</t>
   </si>
   <si>
     <t>relrec.xpt</t>
@@ -368,7 +326,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -399,16 +357,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -439,20 +389,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor rgb="FFD9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="4">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -460,54 +398,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFA5A5A5"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFA5A5A5"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFA5A5A5"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFA5A5A5"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFA5A5A5"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFA5A5A5"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFA5A5A5"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -547,21 +442,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -963,26 +843,26 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
         <v>25</v>
-      </c>
-      <c r="B2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" t="s">
         <v>27</v>
-      </c>
-      <c r="B3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="B4" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1014,10 +894,10 @@
         <v>17</v>
       </c>
       <c r="E1" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" s="9" t="s">
         <v>84</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>85</v>
       </c>
       <c r="G1" s="9" t="s">
         <v>18</v>
@@ -1026,10 +906,10 @@
         <v>19</v>
       </c>
       <c r="I1" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="J1" s="9" t="s">
         <v>86</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>87</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>20</v>
@@ -1038,72 +918,72 @@
         <v>21</v>
       </c>
       <c r="M1" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="N1" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="O1" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="P1" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="O1" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="P1" s="10" t="s">
+      <c r="Q1" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="64" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="P2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="J2" s="2" t="s">
+      <c r="Q2" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="16" x14ac:dyDescent="0.2">
@@ -1173,81 +1053,81 @@
         <v>8</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F4" s="2">
         <v>20</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="N4" s="2">
         <v>8</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="14" t="s">
         <v>57</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>58</v>
       </c>
       <c r="D5" s="6">
         <v>1</v>
       </c>
-      <c r="E5" s="19" t="s">
-        <v>60</v>
+      <c r="E5" s="14" t="s">
+        <v>59</v>
       </c>
       <c r="F5" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="G5" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="H5" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="I5" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="H5" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="I5" s="14" t="s">
-        <v>95</v>
-      </c>
       <c r="J5" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K5" s="6">
         <v>9</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M5" s="6">
         <v>9</v>
@@ -1256,51 +1136,51 @@
         <v>9</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P5" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>57</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>58</v>
       </c>
       <c r="D6" s="6">
         <v>3</v>
       </c>
       <c r="E6" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="H6" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="F6" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="G6" s="13" t="s">
+      <c r="I6" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="H6" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="I6" s="14" t="s">
-        <v>95</v>
-      </c>
       <c r="J6" s="14" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="K6" s="6">
         <v>10</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M6" s="6">
         <v>10</v>
@@ -1309,13 +1189,13 @@
         <v>10</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P6" s="13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Q6" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1352,10 +1232,10 @@
         <v>9</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>10</v>
@@ -1364,7 +1244,7 @@
         <v>11</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>12</v>
@@ -1373,75 +1253,75 @@
         <v>13</v>
       </c>
       <c r="L1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="P1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q1" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="P2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q2" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="16" x14ac:dyDescent="0.2">
@@ -1511,78 +1391,78 @@
         <v>8</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M4" s="2">
         <v>8</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D5" s="6">
         <v>1</v>
       </c>
       <c r="E5" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="G5" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="I5" s="8" t="s">
         <v>62</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>63</v>
       </c>
       <c r="J5" s="6">
         <v>1.87</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L5" s="6">
         <v>1.87</v>
@@ -1591,51 +1471,51 @@
         <v>1.87</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P5" s="6">
         <v>1</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D6" s="6">
         <v>2</v>
       </c>
       <c r="E6" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="F6" s="19" t="s">
-        <v>60</v>
-      </c>
       <c r="G6" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H6" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="6" t="s">
-        <v>66</v>
-      </c>
       <c r="I6" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J6" s="6">
         <v>44.5</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L6" s="6">
         <v>44.5</v>
@@ -1644,51 +1524,51 @@
         <v>44.5</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P6" s="6">
         <v>1</v>
       </c>
       <c r="Q6" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D7" s="6">
         <v>3</v>
       </c>
       <c r="E7" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F7" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="F7" s="19" t="s">
-        <v>60</v>
-      </c>
       <c r="G7" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="H7" s="6" t="s">
-        <v>69</v>
-      </c>
       <c r="I7" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J7" s="6">
         <v>294.7</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="L7" s="6">
         <v>294.7</v>
@@ -1697,51 +1577,51 @@
         <v>294.7</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P7" s="6">
         <v>1</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D8" s="6">
         <v>4</v>
       </c>
       <c r="E8" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="F8" s="19" t="s">
-        <v>60</v>
-      </c>
       <c r="G8" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="H8" s="6" t="s">
-        <v>72</v>
-      </c>
       <c r="I8" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J8" s="6">
         <v>0.75</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L8" s="6">
         <v>0.75</v>
@@ -1750,51 +1630,51 @@
         <v>0.75</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P8" s="6">
         <v>1</v>
       </c>
       <c r="Q8" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D9" s="6">
         <v>5</v>
       </c>
       <c r="E9" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="F9" s="19" t="s">
-        <v>60</v>
-      </c>
       <c r="G9" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H9" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="H9" s="6" t="s">
-        <v>74</v>
-      </c>
       <c r="I9" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J9" s="6">
         <v>4.6900000000000004</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L9" s="6">
         <v>4.6900000000000004</v>
@@ -1803,51 +1683,51 @@
         <v>4.6900000000000004</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P9" s="6">
         <v>1</v>
       </c>
       <c r="Q9" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D10" s="6">
         <v>6</v>
       </c>
       <c r="E10" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="F10" s="19" t="s">
-        <v>60</v>
-      </c>
       <c r="G10" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="H10" s="6" t="s">
-        <v>76</v>
-      </c>
       <c r="I10" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J10" s="6">
         <v>10.9</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L10" s="6">
         <v>10.9</v>
@@ -1856,51 +1736,51 @@
         <v>10.9</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P10" s="6">
         <v>1</v>
       </c>
       <c r="Q10" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D11" s="6">
         <v>7</v>
       </c>
       <c r="E11" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="F11" s="19" t="s">
-        <v>60</v>
-      </c>
       <c r="G11" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="H11" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="6" t="s">
-        <v>79</v>
-      </c>
       <c r="I11" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J11" s="6">
         <v>1.68</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L11" s="6">
         <v>1.68</v>
@@ -1909,51 +1789,51 @@
         <v>1.68</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P11" s="6">
         <v>8</v>
       </c>
       <c r="Q11" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D12" s="6">
         <v>8</v>
       </c>
       <c r="E12" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F12" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="G12" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="I12" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>83</v>
       </c>
       <c r="J12" s="6">
         <v>1.91</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L12" s="6">
         <v>1.91</v>
@@ -1962,51 +1842,51 @@
         <v>1.91</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="P12" s="6">
         <v>8</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D13" s="6">
         <v>9</v>
       </c>
       <c r="E13" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F13" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="G13" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I13" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="I13" s="8" t="s">
-        <v>83</v>
       </c>
       <c r="J13" s="6">
         <v>46</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L13" s="6">
         <v>46</v>
@@ -2015,51 +1895,51 @@
         <v>46</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O13" s="6" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="P13" s="6">
         <v>8</v>
       </c>
       <c r="Q13" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D14" s="6">
         <v>10</v>
       </c>
       <c r="E14" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F14" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="G14" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="I14" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="I14" s="8" t="s">
-        <v>83</v>
       </c>
       <c r="J14" s="6">
         <v>289</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="L14" s="6">
         <v>289</v>
@@ -2068,51 +1948,51 @@
         <v>289</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="P14" s="6">
         <v>8</v>
       </c>
       <c r="Q14" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D15" s="6">
         <v>11</v>
       </c>
       <c r="E15" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F15" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="G15" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="I15" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>83</v>
       </c>
       <c r="J15" s="6">
         <v>0.77</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L15" s="6">
         <v>0.77</v>
@@ -2121,51 +2001,51 @@
         <v>0.77</v>
       </c>
       <c r="N15" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="P15" s="6">
         <v>8</v>
       </c>
       <c r="Q15" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D16" s="6">
         <v>12</v>
       </c>
       <c r="E16" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F16" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="G16" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="I16" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="I16" s="8" t="s">
-        <v>83</v>
       </c>
       <c r="J16" s="6">
         <v>4.5</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L16" s="6">
         <v>4.5</v>
@@ -2174,16 +2054,16 @@
         <v>4.5</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="P16" s="6">
         <v>8</v>
       </c>
       <c r="Q16" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -2194,431 +2074,4 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C2DFA22-7454-AA4B-BC49-0F3BD2B98BB8}">
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="3" max="3" width="14.5" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="C1" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="E1" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="F1" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="G1" s="16" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="48" x14ac:dyDescent="0.2">
-      <c r="A2" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="E2" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="F2" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="G2" s="17" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="18" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>107</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="17" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="13">
-        <v>1</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G5" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="13">
-        <v>1</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G6" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="13">
-        <v>2</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G7" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="13">
-        <v>3</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G8" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="13">
-        <v>4</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G9" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" s="13">
-        <v>5</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G10" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" s="13">
-        <v>6</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G11" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="13">
-        <v>7</v>
-      </c>
-      <c r="F12" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G12" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="13">
-        <v>3</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G13" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" s="13">
-        <v>8</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G14" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" s="13">
-        <v>9</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G15" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E16" s="13">
-        <v>10</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G16" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E17" s="13">
-        <v>11</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G17" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E18" s="13">
-        <v>12</v>
-      </c>
-      <c r="F18" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="G18" s="13">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>